<commit_message>
Refresh POWR TTM_capex KPI export
</commit_message>
<xml_diff>
--- a/buckets/POWR/POWR_kpi.xlsx
+++ b/buckets/POWR/POWR_kpi.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yuuji\Dropbox\Kaissa Consumer\Mosaic\buckets\POWR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{459D5ED1-F0B6-483A-ABEF-DBAFA433DC1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BF7F2A0-CAD4-4160-8CAE-7AEDABE6259E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="21600" yWindow="-16200" windowWidth="19410" windowHeight="15585" activeTab="1" xr2:uid="{30DE43AD-F492-43CF-BD64-FB4AD4D1959C}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="2" xr2:uid="{30DE43AD-F492-43CF-BD64-FB4AD4D1959C}"/>
   </bookViews>
   <sheets>
     <sheet name="AEE" sheetId="1" r:id="rId1"/>
@@ -48,9 +48,8 @@
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
 <metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="2">
+  <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
   <futureMetadata name="XLDAPR" count="1">
     <bk>
@@ -61,35 +60,11 @@
       </extLst>
     </bk>
   </futureMetadata>
-  <futureMetadata name="XLRICHVALUE" count="2">
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="0"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="1"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
   <cellMetadata count="1">
     <bk>
       <rc t="1" v="0"/>
     </bk>
   </cellMetadata>
-  <valueMetadata count="2">
-    <bk>
-      <rc t="2" v="0"/>
-    </bk>
-    <bk>
-      <rc t="2" v="1"/>
-    </bk>
-  </valueMetadata>
 </metadata>
 </file>
 
@@ -487,170 +462,98 @@
       <tp t="s">
         <v>#N/A N/A</v>
         <stp/>
-        <stp>BDH|11113501292731076605</stp>
-        <tr r="D23" s="15"/>
+        <stp>BDH|10666564483243728762</stp>
+        <tr r="D23" s="12"/>
       </tp>
       <tp t="s">
         <v>#N/A N/A</v>
         <stp/>
-        <stp>BDH|11375011732338803024</stp>
-        <tr r="D6" s="1"/>
+        <stp>BDH|10775451014990933921</stp>
+        <tr r="D14" s="12"/>
       </tp>
       <tp t="s">
         <v>#N/A N/A</v>
         <stp/>
-        <stp>BDH|15000901654646701748</stp>
-        <tr r="D14" s="1"/>
+        <stp>BDH|15977772103892996216</stp>
+        <tr r="D6" s="12"/>
       </tp>
       <tp t="s">
         <v>#N/A N/A</v>
         <stp/>
-        <stp>BDH|11603849834027454179</stp>
-        <tr r="D6" s="13"/>
-      </tp>
-      <tp t="s">
-        <v>#N/A N/A</v>
-        <stp/>
-        <stp>BDH|12095955190868836621</stp>
-        <tr r="D6" s="15"/>
-      </tp>
-      <tp t="s">
-        <v>#N/A N/A</v>
-        <stp/>
-        <stp>BDH|18179939496851995865</stp>
-        <tr r="D14" s="14"/>
-      </tp>
-      <tp t="s">
-        <v>#N/A N/A</v>
-        <stp/>
-        <stp>BDH|16727857878568693797</stp>
-        <tr r="D6" s="14"/>
-      </tp>
-      <tp t="s">
-        <v>#N/A N/A</v>
-        <stp/>
-        <stp>BDH|15758173608431013089</stp>
-        <tr r="D23" s="12"/>
+        <stp>BDH|15597115716912653397</stp>
+        <tr r="D14" s="15"/>
       </tp>
     </main>
     <main first="bofaddin.rtdserver">
       <tp t="s">
         <v>#N/A N/A</v>
         <stp/>
-        <stp>BDH|6786892725102373248</stp>
-        <tr r="D14" s="12"/>
+        <stp>BDH|6045638057872329849</stp>
+        <tr r="D23" s="1"/>
       </tp>
-    </main>
-    <main first="bofaddin.rtdserver">
       <tp t="s">
         <v>#N/A N/A</v>
         <stp/>
-        <stp>BDH|7434619623679670068</stp>
+        <stp>BDH|1899021169798102057</stp>
+        <tr r="D6" s="13"/>
+      </tp>
+      <tp t="s">
+        <v>#N/A N/A</v>
+        <stp/>
+        <stp>BDH|5853901973542797079</stp>
+        <tr r="D14" s="1"/>
+      </tp>
+      <tp t="s">
+        <v>#N/A N/A</v>
+        <stp/>
+        <stp>BDH|2867808584084623235</stp>
+        <tr r="D14" s="14"/>
+      </tp>
+      <tp t="s">
+        <v>#N/A N/A</v>
+        <stp/>
+        <stp>BDH|6709661677442251181</stp>
+        <tr r="D23" s="13"/>
+      </tp>
+      <tp t="s">
+        <v>#N/A N/A</v>
+        <stp/>
+        <stp>BDH|5622626010393012459</stp>
+        <tr r="D6" s="14"/>
+      </tp>
+      <tp t="s">
+        <v>#N/A N/A</v>
+        <stp/>
+        <stp>BDH|8934810464407397018</stp>
+        <tr r="D14" s="13"/>
+      </tp>
+      <tp t="s">
+        <v>#N/A N/A</v>
+        <stp/>
+        <stp>BDH|4250969443298994371</stp>
+        <tr r="D6" s="1"/>
+      </tp>
+      <tp t="s">
+        <v>#N/A N/A</v>
+        <stp/>
+        <stp>BDH|8302811472737330209</stp>
         <tr r="D23" s="14"/>
       </tp>
       <tp t="s">
         <v>#N/A N/A</v>
         <stp/>
-        <stp>BDH|2189126329492519640</stp>
-        <tr r="D23" s="13"/>
+        <stp>BDH|6579188173574972772</stp>
+        <tr r="D23" s="15"/>
       </tp>
       <tp t="s">
         <v>#N/A N/A</v>
         <stp/>
-        <stp>BDH|1969007940541391132</stp>
-        <tr r="D23" s="1"/>
-      </tp>
-      <tp t="s">
-        <v>#N/A N/A</v>
-        <stp/>
-        <stp>BDH|7557388571286783558</stp>
-        <tr r="D14" s="15"/>
-      </tp>
-      <tp t="s">
-        <v>#N/A N/A</v>
-        <stp/>
-        <stp>BDH|2704080548460421423</stp>
-        <tr r="D6" s="12"/>
-      </tp>
-      <tp t="s">
-        <v>#N/A N/A</v>
-        <stp/>
-        <stp>BDH|380970110915663384</stp>
-        <tr r="D14" s="13"/>
+        <stp>BDH|132837973015176345</stp>
+        <tr r="D6" s="15"/>
       </tp>
     </main>
   </volType>
 </volTypes>
-</file>
-
-<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
-<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
-  <global>
-    <keyFlags>
-      <key name="_Self">
-        <flag name="ExcludeFromFile" value="1"/>
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_DisplayString">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Flags">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Format">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_SubLabel">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Attribution">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Icon">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Display">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_CanonicalPropertyNames">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_ClassificationId">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-    </keyFlags>
-  </global>
-</rvTypesInfo>
-</file>
-
-<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="2">
-  <rv s="0">
-    <v>756</v>
-    <v>8</v>
-    <v>0</v>
-    <v>1</v>
-  </rv>
-  <rv s="1">
-    <v>8</v>
-    <v>1</v>
-  </rv>
-</rvData>
-</file>
-
-<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
-<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="2">
-  <s t="_error">
-    <k n="colOffset" t="i"/>
-    <k n="errorType" t="i"/>
-    <k n="rwOffset" t="i"/>
-    <k n="subType" t="i"/>
-  </s>
-  <s t="_error">
-    <k n="errorType" t="i"/>
-    <k n="propagated" t="b"/>
-  </s>
-</rvStructures>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1138,7 +1041,7 @@
       </c>
       <c r="B3" s="19">
         <f ca="1">+B4-365*3</f>
-        <v>44991</v>
+        <v>45001</v>
       </c>
       <c r="Q3" s="24" t="str">
         <f ca="1"/>
@@ -1183,7 +1086,7 @@
       </c>
       <c r="B4" s="21">
         <f ca="1">TODAY()</f>
-        <v>46086</v>
+        <v>46096</v>
       </c>
       <c r="Q4" s="24" t="str">
         <f ca="1"/>
@@ -1714,23 +1617,23 @@
       </c>
       <c r="U10" s="30" t="str">
         <f ca="1"/>
-        <v/>
-      </c>
-      <c r="V10" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="W10" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="X10" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Y10" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
+        <v>4620</v>
+      </c>
+      <c r="V10" s="29" t="str">
+        <f ca="1"/>
+        <v>0.235294117647059</v>
+      </c>
+      <c r="W10" s="29" t="str">
+        <f ca="1"/>
+        <v>685.835566778728</v>
+      </c>
+      <c r="X10" s="29" t="str">
+        <f ca="1"/>
+        <v>1850.27338652394</v>
+      </c>
+      <c r="Y10" s="29" t="str">
+        <f ca="1"/>
+        <v>0.0428893905191874</v>
       </c>
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.45">
@@ -1772,23 +1675,23 @@
       </c>
       <c r="U11" s="30" t="str">
         <f ca="1"/>
-        <v/>
-      </c>
-      <c r="V11" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="W11" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="X11" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Y11" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
+        <v>4657</v>
+      </c>
+      <c r="V11" s="29" t="str">
+        <f ca="1"/>
+        <v>0.208982346832814</v>
+      </c>
+      <c r="W11" s="29" t="str">
+        <f ca="1"/>
+        <v>-263.117708142449</v>
+      </c>
+      <c r="X11" s="29" t="str">
+        <f ca="1"/>
+        <v>1715.46311282047</v>
+      </c>
+      <c r="Y11" s="29" t="str">
+        <f ca="1"/>
+        <v>0.00800865800865802</v>
       </c>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.45">
@@ -1810,23 +1713,23 @@
       </c>
       <c r="U12" s="30" t="str">
         <f ca="1"/>
-        <v/>
-      </c>
-      <c r="V12" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="W12" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="X12" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Y12" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
+        <v>4488</v>
+      </c>
+      <c r="V12" s="29" t="str">
+        <f ca="1"/>
+        <v>0.0564971751412429</v>
+      </c>
+      <c r="W12" s="29" t="str">
+        <f ca="1"/>
+        <v>-1524.85171691571</v>
+      </c>
+      <c r="X12" s="29" t="str">
+        <f ca="1"/>
+        <v>-1317.54573110505</v>
+      </c>
+      <c r="Y12" s="29" t="str">
+        <f ca="1"/>
+        <v>-0.0362894567318016</v>
       </c>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.45">
@@ -1899,23 +1802,23 @@
       </c>
       <c r="U13" s="30" t="str">
         <f ca="1"/>
-        <v/>
-      </c>
-      <c r="V13" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="W13" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="X13" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Y13" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
+        <v>3318</v>
+      </c>
+      <c r="V13" s="29" t="str">
+        <f ca="1"/>
+        <v>-0.251015801354402</v>
+      </c>
+      <c r="W13" s="29" t="str">
+        <f ca="1"/>
+        <v>-3075.12976495645</v>
+      </c>
+      <c r="X13" s="29" t="str">
+        <f ca="1"/>
+        <v>-4177.26362323588</v>
+      </c>
+      <c r="Y13" s="29" t="str">
+        <f ca="1"/>
+        <v>-0.260695187165775</v>
       </c>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.45">
@@ -2527,20 +2430,54 @@
       <c r="C23" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D23" s="3" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="D23" ca="1">-_xll.BDH($B$2,C23,$B$3,$B$4,"DIR=H","DATES=H")</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E23" s="3"/>
-      <c r="F23" s="3"/>
-      <c r="G23" s="3"/>
-      <c r="H23" s="3"/>
-      <c r="I23" s="3"/>
-      <c r="J23" s="3"/>
-      <c r="K23" s="3"/>
-      <c r="L23" s="3"/>
-      <c r="M23" s="3"/>
-      <c r="N23" s="3"/>
+      <c r="D23" s="3" cm="1">
+        <f t="array" aca="1" ref="D23:O23" ca="1">-_xll.BDH($B$2,C23,$B$3,$B$4,"DIR=H","DATES=H")</f>
+        <v>3561</v>
+      </c>
+      <c r="E23" s="3">
+        <f ca="1"/>
+        <v>3713</v>
+      </c>
+      <c r="F23" s="3">
+        <f ca="1"/>
+        <v>3575</v>
+      </c>
+      <c r="G23" s="3">
+        <f ca="1"/>
+        <v>3797</v>
+      </c>
+      <c r="H23" s="3">
+        <f ca="1"/>
+        <v>3740</v>
+      </c>
+      <c r="I23" s="3">
+        <f ca="1"/>
+        <v>3852</v>
+      </c>
+      <c r="J23" s="3">
+        <f ca="1"/>
+        <v>4248</v>
+      </c>
+      <c r="K23" s="3">
+        <f ca="1"/>
+        <v>4430</v>
+      </c>
+      <c r="L23" s="3">
+        <f ca="1"/>
+        <v>4620</v>
+      </c>
+      <c r="M23" s="3">
+        <f ca="1"/>
+        <v>4657</v>
+      </c>
+      <c r="N23" s="3">
+        <f ca="1"/>
+        <v>4488</v>
+      </c>
+      <c r="O23">
+        <f ca="1"/>
+        <v>3318</v>
+      </c>
       <c r="Q23" s="24" t="str">
         <v>AEE US EQUITY</v>
       </c>
@@ -2577,37 +2514,37 @@
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
-      <c r="H24" s="12" t="e" vm="2">
+      <c r="H24" s="12">
         <f t="shared" ref="H24" ca="1" si="10">+H23/D23-1</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="I24" s="12" t="e">
-        <f t="shared" ref="I24" si="11">+I23/E23-1</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J24" s="12" t="e">
-        <f t="shared" ref="J24" si="12">+J23/F23-1</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K24" s="12" t="e">
-        <f t="shared" ref="K24" si="13">+K23/G23-1</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L24" s="12" t="e">
-        <f t="shared" ref="L24" si="14">+L23/H23-1</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M24" s="12" t="e">
-        <f t="shared" ref="M24" si="15">+M23/I23-1</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N24" s="12" t="e">
-        <f t="shared" ref="N24" si="16">+N23/J23-1</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O24" s="12" t="e">
-        <f t="shared" ref="O24" si="17">+O23/K23-1</f>
-        <v>#DIV/0!</v>
+        <v>5.0266778994664474E-2</v>
+      </c>
+      <c r="I24" s="12">
+        <f t="shared" ref="I24" ca="1" si="11">+I23/E23-1</f>
+        <v>3.7436035550767466E-2</v>
+      </c>
+      <c r="J24" s="12">
+        <f t="shared" ref="J24" ca="1" si="12">+J23/F23-1</f>
+        <v>0.18825174825174829</v>
+      </c>
+      <c r="K24" s="12">
+        <f t="shared" ref="K24" ca="1" si="13">+K23/G23-1</f>
+        <v>0.16671056096918613</v>
+      </c>
+      <c r="L24" s="12">
+        <f t="shared" ref="L24" ca="1" si="14">+L23/H23-1</f>
+        <v>0.23529411764705888</v>
+      </c>
+      <c r="M24" s="12">
+        <f t="shared" ref="M24" ca="1" si="15">+M23/I23-1</f>
+        <v>0.20898234683281403</v>
+      </c>
+      <c r="N24" s="12">
+        <f t="shared" ref="N24" ca="1" si="16">+N23/J23-1</f>
+        <v>5.6497175141242861E-2</v>
+      </c>
+      <c r="O24" s="12">
+        <f t="shared" ref="O24" ca="1" si="17">+O23/K23-1</f>
+        <v>-0.25101580135440182</v>
       </c>
       <c r="Q24" s="24" t="str">
         <v>AEE US EQUITY</v>
@@ -2642,21 +2579,21 @@
         <v>13</v>
       </c>
       <c r="D25" s="1"/>
-      <c r="L25" s="7" t="e">
-        <f>(L24-K24)*10000</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M25" s="7" t="e">
-        <f>(M24-L24)*10000</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N25" s="7" t="e">
-        <f>(N24-M24)*10000</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O25" s="7" t="e">
-        <f>(O24-N24)*10000</f>
-        <v>#DIV/0!</v>
+      <c r="L25" s="7">
+        <f ca="1">(L24-K24)*10000</f>
+        <v>685.83556677872753</v>
+      </c>
+      <c r="M25" s="7">
+        <f ca="1">(M24-L24)*10000</f>
+        <v>-263.11770814244852</v>
+      </c>
+      <c r="N25" s="7">
+        <f ca="1">(N24-M24)*10000</f>
+        <v>-1524.8517169157117</v>
+      </c>
+      <c r="O25" s="7">
+        <f ca="1">(O24-N24)*10000</f>
+        <v>-3075.1297649564467</v>
       </c>
       <c r="Q25" s="24" t="str">
         <v>AEE US EQUITY</v>
@@ -2698,21 +2635,21 @@
       <c r="I26" s="6"/>
       <c r="J26" s="6"/>
       <c r="K26" s="6"/>
-      <c r="L26" s="7" t="e">
+      <c r="L26" s="7">
         <f ca="1">(L24-H24)*10000</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M26" s="7" t="e">
-        <f>(M24-I24)*10000</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N26" s="7" t="e">
-        <f>(N24-J24)*10000</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O26" s="7" t="e">
-        <f>(O24-K24)*10000</f>
-        <v>#DIV/0!</v>
+        <v>1850.2733865239441</v>
+      </c>
+      <c r="M26" s="7">
+        <f ca="1">(M24-I24)*10000</f>
+        <v>1715.4631128204655</v>
+      </c>
+      <c r="N26" s="7">
+        <f ca="1">(N24-J24)*10000</f>
+        <v>-1317.5457311050543</v>
+      </c>
+      <c r="O26" s="7">
+        <f ca="1">(O24-K24)*10000</f>
+        <v>-4177.2636232358791</v>
       </c>
       <c r="Q26" s="24" t="str" cm="1">
         <f t="array" ref="Q26:Y29">_xlfn.LET(
@@ -2767,21 +2704,21 @@
         <v>4</v>
       </c>
       <c r="D27" s="1"/>
-      <c r="L27" s="12" t="e">
-        <f t="shared" ref="L27" si="18">L23/K23-1</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M27" s="12" t="e">
-        <f t="shared" ref="M27" si="19">M23/L23-1</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N27" s="12" t="e">
-        <f t="shared" ref="N27" si="20">N23/M23-1</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O27" s="12" t="e">
-        <f t="shared" ref="O27" si="21">O23/N23-1</f>
-        <v>#DIV/0!</v>
+      <c r="L27" s="12">
+        <f t="shared" ref="L27" ca="1" si="18">L23/K23-1</f>
+        <v>4.2889390519187387E-2</v>
+      </c>
+      <c r="M27" s="12">
+        <f t="shared" ref="M27" ca="1" si="19">M23/L23-1</f>
+        <v>8.0086580086580206E-3</v>
+      </c>
+      <c r="N27" s="12">
+        <f t="shared" ref="N27" ca="1" si="20">N23/M23-1</f>
+        <v>-3.6289456731801617E-2</v>
+      </c>
+      <c r="O27" s="12">
+        <f t="shared" ref="O27" ca="1" si="21">O23/N23-1</f>
+        <v>-0.26069518716577544</v>
       </c>
       <c r="Q27" s="24" t="str">
         <v>AEE US EQUITY</v>
@@ -3790,7 +3727,7 @@
       </c>
       <c r="B3" s="19">
         <f ca="1">+B4-365*3</f>
-        <v>44991</v>
+        <v>45001</v>
       </c>
       <c r="Q3" s="24" t="str">
         <f ca="1"/>
@@ -3835,7 +3772,7 @@
       </c>
       <c r="B4" s="21">
         <f ca="1">TODAY()</f>
-        <v>46086</v>
+        <v>46096</v>
       </c>
       <c r="Q4" s="24" t="str">
         <f ca="1"/>
@@ -4366,23 +4303,23 @@
       </c>
       <c r="U10" s="30" t="str">
         <f ca="1"/>
-        <v/>
-      </c>
-      <c r="V10" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="W10" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="X10" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Y10" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
+        <v>8111.2</v>
+      </c>
+      <c r="V10" s="29" t="str">
+        <f ca="1"/>
+        <v>0.124977462171121</v>
+      </c>
+      <c r="W10" s="29" t="str">
+        <f ca="1"/>
+        <v>897.946206337867</v>
+      </c>
+      <c r="X10" s="29" t="str">
+        <f ca="1"/>
+        <v>1160.78000896371</v>
+      </c>
+      <c r="Y10" s="29" t="str">
+        <f ca="1"/>
+        <v>0.0438318791341723</v>
       </c>
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.45">
@@ -4424,23 +4361,23 @@
       </c>
       <c r="U11" s="30" t="str">
         <f ca="1"/>
-        <v/>
-      </c>
-      <c r="V11" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="W11" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="X11" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Y11" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
+        <v>8448.3</v>
+      </c>
+      <c r="V11" s="29" t="str">
+        <f ca="1"/>
+        <v>0.247718210013292</v>
+      </c>
+      <c r="W11" s="29" t="str">
+        <f ca="1"/>
+        <v>1227.40747842171</v>
+      </c>
+      <c r="X11" s="29" t="str">
+        <f ca="1"/>
+        <v>3672.46960891032</v>
+      </c>
+      <c r="Y11" s="29" t="str">
+        <f ca="1"/>
+        <v>0.0415598185225368</v>
       </c>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.45">
@@ -4462,23 +4399,23 @@
       </c>
       <c r="U12" s="30" t="str">
         <f ca="1"/>
-        <v/>
-      </c>
-      <c r="V12" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="W12" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="X12" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Y12" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
+        <v>8593.7</v>
+      </c>
+      <c r="V12" s="29" t="str">
+        <f ca="1"/>
+        <v>0.237304729681089</v>
+      </c>
+      <c r="W12" s="29" t="str">
+        <f ca="1"/>
+        <v>-104.134803322034</v>
+      </c>
+      <c r="X12" s="29" t="str">
+        <f ca="1"/>
+        <v>3422.66069887274</v>
+      </c>
+      <c r="Y12" s="29" t="str">
+        <f ca="1"/>
+        <v>0.0172105630718609</v>
       </c>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.45">
@@ -4551,23 +4488,23 @@
       </c>
       <c r="U13" s="30" t="str">
         <f ca="1"/>
-        <v/>
-      </c>
-      <c r="V13" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="W13" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="X13" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Y13" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
+        <v>8583</v>
+      </c>
+      <c r="V13" s="29" t="str">
+        <f ca="1"/>
+        <v>0.104547911358196</v>
+      </c>
+      <c r="W13" s="29" t="str">
+        <f ca="1"/>
+        <v>-1327.56818322892</v>
+      </c>
+      <c r="X13" s="29" t="str">
+        <f ca="1"/>
+        <v>693.650698208619</v>
+      </c>
+      <c r="Y13" s="29" t="str">
+        <f ca="1"/>
+        <v>-0.00124509815329843</v>
       </c>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.45">
@@ -5179,20 +5116,54 @@
       <c r="C23" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D23" s="3" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="D23" ca="1">-_xll.BDH($B$2,C23,$B$3,$B$4,"DIR=H","DATES=H")</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E23" s="3"/>
-      <c r="F23" s="3"/>
-      <c r="G23" s="3"/>
-      <c r="H23" s="3"/>
-      <c r="I23" s="3"/>
-      <c r="J23" s="3"/>
-      <c r="K23" s="3"/>
-      <c r="L23" s="3"/>
-      <c r="M23" s="3"/>
-      <c r="N23" s="3"/>
+      <c r="D23" s="3" cm="1">
+        <f t="array" aca="1" ref="D23:O23" ca="1">-_xll.BDH($B$2,C23,$B$3,$B$4,"DIR=H","DATES=H")</f>
+        <v>7146.5</v>
+      </c>
+      <c r="E23" s="3">
+        <f ca="1"/>
+        <v>7690.2</v>
+      </c>
+      <c r="F23" s="3">
+        <f ca="1"/>
+        <v>7760</v>
+      </c>
+      <c r="G23" s="3">
+        <f ca="1"/>
+        <v>7506.5</v>
+      </c>
+      <c r="H23" s="3">
+        <f ca="1"/>
+        <v>7210.1</v>
+      </c>
+      <c r="I23" s="3">
+        <f ca="1"/>
+        <v>6771</v>
+      </c>
+      <c r="J23" s="3">
+        <f ca="1"/>
+        <v>6945.5</v>
+      </c>
+      <c r="K23" s="3">
+        <f ca="1"/>
+        <v>7770.6</v>
+      </c>
+      <c r="L23" s="3">
+        <f ca="1"/>
+        <v>8111.2</v>
+      </c>
+      <c r="M23" s="3">
+        <f ca="1"/>
+        <v>8448.2999999999993</v>
+      </c>
+      <c r="N23" s="3">
+        <f ca="1"/>
+        <v>8593.7000000000007</v>
+      </c>
+      <c r="O23">
+        <f ca="1"/>
+        <v>8583</v>
+      </c>
       <c r="Q23" s="24" t="str">
         <v>AEP US EQUITY</v>
       </c>
@@ -5229,37 +5200,37 @@
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
-      <c r="H24" s="12" t="e" vm="2">
+      <c r="H24" s="12">
         <f t="shared" ref="H24:O24" ca="1" si="7">+H23/D23-1</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="I24" s="12" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J24" s="12" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K24" s="12" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L24" s="12" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M24" s="12" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N24" s="12" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O24" s="12" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
+        <v>8.8994612747499424E-3</v>
+      </c>
+      <c r="I24" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>-0.11952875087774051</v>
+      </c>
+      <c r="J24" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>-0.10496134020618553</v>
+      </c>
+      <c r="K24" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>3.5182841537334308E-2</v>
+      </c>
+      <c r="L24" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>0.12497746217112105</v>
+      </c>
+      <c r="M24" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>0.24771821001329197</v>
+      </c>
+      <c r="N24" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>0.23730472968108862</v>
+      </c>
+      <c r="O24" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>0.10454791135819619</v>
       </c>
       <c r="Q24" s="24" t="str">
         <v>AEP US EQUITY</v>
@@ -5294,21 +5265,21 @@
         <v>13</v>
       </c>
       <c r="D25" s="1"/>
-      <c r="L25" s="7" t="e">
-        <f>(L24-K24)*10000</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M25" s="7" t="e">
-        <f>(M24-L24)*10000</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N25" s="7" t="e">
-        <f>(N24-M24)*10000</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O25" s="7" t="e">
-        <f>(O24-N24)*10000</f>
-        <v>#DIV/0!</v>
+      <c r="L25" s="7">
+        <f ca="1">(L24-K24)*10000</f>
+        <v>897.94620633786735</v>
+      </c>
+      <c r="M25" s="7">
+        <f ca="1">(M24-L24)*10000</f>
+        <v>1227.4074784217094</v>
+      </c>
+      <c r="N25" s="7">
+        <f ca="1">(N24-M24)*10000</f>
+        <v>-104.13480332203351</v>
+      </c>
+      <c r="O25" s="7">
+        <f ca="1">(O24-N24)*10000</f>
+        <v>-1327.5681832289242</v>
       </c>
       <c r="Q25" s="24" t="str">
         <v>AEP US EQUITY</v>
@@ -5350,21 +5321,21 @@
       <c r="I26" s="6"/>
       <c r="J26" s="6"/>
       <c r="K26" s="6"/>
-      <c r="L26" s="7" t="e">
+      <c r="L26" s="7">
         <f ca="1">(L24-H24)*10000</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M26" s="7" t="e">
-        <f>(M24-I24)*10000</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N26" s="7" t="e">
-        <f>(N24-J24)*10000</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O26" s="7" t="e">
-        <f>(O24-K24)*10000</f>
-        <v>#DIV/0!</v>
+        <v>1160.780008963711</v>
+      </c>
+      <c r="M26" s="7">
+        <f ca="1">(M24-I24)*10000</f>
+        <v>3672.469608910325</v>
+      </c>
+      <c r="N26" s="7">
+        <f ca="1">(N24-J24)*10000</f>
+        <v>3422.6606988727417</v>
+      </c>
+      <c r="O26" s="7">
+        <f ca="1">(O24-K24)*10000</f>
+        <v>693.65069820861879</v>
       </c>
       <c r="Q26" s="24" t="str" cm="1">
         <f t="array" ref="Q26:Y29">_xlfn.LET(
@@ -5419,21 +5390,21 @@
         <v>4</v>
       </c>
       <c r="D27" s="1"/>
-      <c r="L27" s="12" t="e">
-        <f t="shared" ref="L27:O27" si="8">L23/K23-1</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M27" s="12" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N27" s="12" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O27" s="12" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
+      <c r="L27" s="12">
+        <f t="shared" ref="L27:O27" ca="1" si="8">L23/K23-1</f>
+        <v>4.3831879134172302E-2</v>
+      </c>
+      <c r="M27" s="12">
+        <f t="shared" ca="1" si="8"/>
+        <v>4.1559818522536762E-2</v>
+      </c>
+      <c r="N27" s="12">
+        <f t="shared" ca="1" si="8"/>
+        <v>1.7210563071860863E-2</v>
+      </c>
+      <c r="O27" s="12">
+        <f t="shared" ca="1" si="8"/>
+        <v>-1.2450981532984295E-3</v>
       </c>
       <c r="Q27" s="24" t="str">
         <v>AEP US EQUITY</v>
@@ -6425,7 +6396,7 @@
       </c>
       <c r="B3" s="19">
         <f ca="1">+B4-365*3</f>
-        <v>44991</v>
+        <v>45001</v>
       </c>
       <c r="Q3" s="24" t="str">
         <f ca="1"/>
@@ -6470,7 +6441,7 @@
       </c>
       <c r="B4" s="21">
         <f ca="1">TODAY()</f>
-        <v>46086</v>
+        <v>46096</v>
       </c>
       <c r="Q4" s="24" t="str">
         <f ca="1"/>
@@ -7001,23 +6972,23 @@
       </c>
       <c r="U10" s="30" t="str">
         <f ca="1"/>
-        <v/>
-      </c>
-      <c r="V10" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="W10" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="X10" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Y10" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
+        <v>5901.455</v>
+      </c>
+      <c r="V10" s="29" t="str">
+        <f ca="1"/>
+        <v>0.260930264458717</v>
+      </c>
+      <c r="W10" s="29" t="str">
+        <f ca="1"/>
+        <v>1810.0247539483</v>
+      </c>
+      <c r="X10" s="29" t="str">
+        <f ca="1"/>
+        <v>3332.63562048314</v>
+      </c>
+      <c r="Y10" s="29" t="str">
+        <f ca="1"/>
+        <v>0.126940078946559</v>
       </c>
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.45">
@@ -7059,23 +7030,23 @@
       </c>
       <c r="U11" s="30" t="str">
         <f ca="1"/>
-        <v/>
-      </c>
-      <c r="V11" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="W11" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="X11" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Y11" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
+        <v>6766.953</v>
+      </c>
+      <c r="V11" s="29" t="str">
+        <f ca="1"/>
+        <v>0.453314705920253</v>
+      </c>
+      <c r="W11" s="29" t="str">
+        <f ca="1"/>
+        <v>1923.84441461536</v>
+      </c>
+      <c r="X11" s="29" t="str">
+        <f ca="1"/>
+        <v>5080.39033843952</v>
+      </c>
+      <c r="Y11" s="29" t="str">
+        <f ca="1"/>
+        <v>0.146658408816131</v>
       </c>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.45">
@@ -7097,23 +7068,23 @@
       </c>
       <c r="U12" s="30" t="str">
         <f ca="1"/>
-        <v/>
-      </c>
-      <c r="V12" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="W12" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="X12" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Y12" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
+        <v>6979.859</v>
+      </c>
+      <c r="V12" s="29" t="str">
+        <f ca="1"/>
+        <v>0.328602107228351</v>
+      </c>
+      <c r="W12" s="29" t="str">
+        <f ca="1"/>
+        <v>-1247.12598691902</v>
+      </c>
+      <c r="X12" s="29" t="str">
+        <f ca="1"/>
+        <v>2590.29355198955</v>
+      </c>
+      <c r="Y12" s="29" t="str">
+        <f ca="1"/>
+        <v>0.0314626095378525</v>
       </c>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.45">
@@ -7186,23 +7157,23 @@
       </c>
       <c r="U13" s="30" t="str">
         <f ca="1"/>
-        <v/>
-      </c>
-      <c r="V13" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="W13" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="X13" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Y13" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
+        <v>8070.245</v>
+      </c>
+      <c r="V13" s="29" t="str">
+        <f ca="1"/>
+        <v>0.541091567658836</v>
+      </c>
+      <c r="W13" s="29" t="str">
+        <f ca="1"/>
+        <v>2124.89460430485</v>
+      </c>
+      <c r="X13" s="29" t="str">
+        <f ca="1"/>
+        <v>4611.63778594949</v>
+      </c>
+      <c r="Y13" s="29" t="str">
+        <f ca="1"/>
+        <v>0.156218915023928</v>
       </c>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.45">
@@ -7814,20 +7785,54 @@
       <c r="C23" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D23" s="3" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="D23" ca="1">-_xll.BDH($B$2,C23,$B$3,$B$4,"DIR=H","DATES=H")</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E23" s="3"/>
-      <c r="F23" s="3"/>
-      <c r="G23" s="3"/>
-      <c r="H23" s="3"/>
-      <c r="I23" s="3"/>
-      <c r="J23" s="3"/>
-      <c r="K23" s="3"/>
-      <c r="L23" s="3"/>
-      <c r="M23" s="3"/>
-      <c r="N23" s="3"/>
+      <c r="D23" s="3" cm="1">
+        <f t="array" aca="1" ref="D23:O23" ca="1">-_xll.BDH($B$2,C23,$B$3,$B$4,"DIR=H","DATES=H")</f>
+        <v>5045.1729999999998</v>
+      </c>
+      <c r="E23" s="3">
+        <f ca="1"/>
+        <v>4925.78</v>
+      </c>
+      <c r="F23" s="3">
+        <f ca="1"/>
+        <v>4911.808</v>
+      </c>
+      <c r="G23" s="3">
+        <f ca="1"/>
+        <v>4849.1270000000004</v>
+      </c>
+      <c r="H23" s="3">
+        <f ca="1"/>
+        <v>4680.2389999999996</v>
+      </c>
+      <c r="I23" s="3">
+        <f ca="1"/>
+        <v>4656.22</v>
+      </c>
+      <c r="J23" s="3">
+        <f ca="1"/>
+        <v>5253.5360000000001</v>
+      </c>
+      <c r="K23" s="3">
+        <f ca="1"/>
+        <v>5236.7070000000003</v>
+      </c>
+      <c r="L23" s="3">
+        <f ca="1"/>
+        <v>5901.4549999999999</v>
+      </c>
+      <c r="M23" s="3">
+        <f ca="1"/>
+        <v>6766.9530000000004</v>
+      </c>
+      <c r="N23" s="3">
+        <f ca="1"/>
+        <v>6979.8590000000004</v>
+      </c>
+      <c r="O23">
+        <f ca="1"/>
+        <v>8070.2449999999999</v>
+      </c>
       <c r="Q23" s="24" t="str">
         <v>ETR US EQUITY</v>
       </c>
@@ -7864,37 +7869,37 @@
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
-      <c r="H24" s="12" t="e" vm="2">
+      <c r="H24" s="12">
         <f t="shared" ref="H24:O24" ca="1" si="7">+H23/D23-1</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="I24" s="12" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J24" s="12" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K24" s="12" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L24" s="12" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M24" s="12" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N24" s="12" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O24" s="12" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
+        <v>-7.2333297589597056E-2</v>
+      </c>
+      <c r="I24" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>-5.4724327923699301E-2</v>
+      </c>
+      <c r="J24" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>6.957275202939539E-2</v>
+      </c>
+      <c r="K24" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>7.99277890638872E-2</v>
+      </c>
+      <c r="L24" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>0.26093026445871681</v>
+      </c>
+      <c r="M24" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>0.45331470592025291</v>
+      </c>
+      <c r="N24" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>0.3286021072283507</v>
+      </c>
+      <c r="O24" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>0.54109156765883593</v>
       </c>
       <c r="Q24" s="24" t="str">
         <v>ETR US EQUITY</v>
@@ -7929,21 +7934,21 @@
         <v>13</v>
       </c>
       <c r="D25" s="1"/>
-      <c r="L25" s="7" t="e">
-        <f>(L24-K24)*10000</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M25" s="7" t="e">
-        <f>(M24-L24)*10000</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N25" s="7" t="e">
-        <f>(N24-M24)*10000</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O25" s="7" t="e">
-        <f>(O24-N24)*10000</f>
-        <v>#DIV/0!</v>
+      <c r="L25" s="7">
+        <f ca="1">(L24-K24)*10000</f>
+        <v>1810.0247539482962</v>
+      </c>
+      <c r="M25" s="7">
+        <f ca="1">(M24-L24)*10000</f>
+        <v>1923.8444146153611</v>
+      </c>
+      <c r="N25" s="7">
+        <f ca="1">(N24-M24)*10000</f>
+        <v>-1247.1259869190221</v>
+      </c>
+      <c r="O25" s="7">
+        <f ca="1">(O24-N24)*10000</f>
+        <v>2124.8946043048522</v>
       </c>
       <c r="Q25" s="24" t="str">
         <v>ETR US EQUITY</v>
@@ -7985,21 +7990,21 @@
       <c r="I26" s="6"/>
       <c r="J26" s="6"/>
       <c r="K26" s="6"/>
-      <c r="L26" s="7" t="e">
+      <c r="L26" s="7">
         <f ca="1">(L24-H24)*10000</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M26" s="7" t="e">
-        <f>(M24-I24)*10000</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N26" s="7" t="e">
-        <f>(N24-J24)*10000</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O26" s="7" t="e">
-        <f>(O24-K24)*10000</f>
-        <v>#DIV/0!</v>
+        <v>3332.6356204831386</v>
+      </c>
+      <c r="M26" s="7">
+        <f ca="1">(M24-I24)*10000</f>
+        <v>5080.3903384395226</v>
+      </c>
+      <c r="N26" s="7">
+        <f ca="1">(N24-J24)*10000</f>
+        <v>2590.2935519895532</v>
+      </c>
+      <c r="O26" s="7">
+        <f ca="1">(O24-K24)*10000</f>
+        <v>4611.6377859494869</v>
       </c>
       <c r="Q26" s="24" t="str" cm="1">
         <f t="array" ref="Q26:Y29">_xlfn.LET(
@@ -8054,21 +8059,21 @@
         <v>4</v>
       </c>
       <c r="D27" s="1"/>
-      <c r="L27" s="12" t="e">
-        <f>L23/K23-1</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M27" s="12" t="e">
-        <f>M23/L23-1</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N27" s="12" t="e">
-        <f>N23/M23-1</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O27" s="12" t="e">
-        <f>O23/N23-1</f>
-        <v>#DIV/0!</v>
+      <c r="L27" s="12">
+        <f ca="1">L23/K23-1</f>
+        <v>0.12694007894655934</v>
+      </c>
+      <c r="M27" s="12">
+        <f ca="1">M23/L23-1</f>
+        <v>0.14665840881613113</v>
+      </c>
+      <c r="N27" s="12">
+        <f ca="1">N23/M23-1</f>
+        <v>3.1462609537852515E-2</v>
+      </c>
+      <c r="O27" s="12">
+        <f ca="1">O23/N23-1</f>
+        <v>0.15621891502392815</v>
       </c>
       <c r="Q27" s="24" t="str">
         <v>ETR US EQUITY</v>
@@ -8890,7 +8895,7 @@
       </c>
       <c r="B3" s="19">
         <f ca="1">+B4-365*3</f>
-        <v>44991</v>
+        <v>45001</v>
       </c>
       <c r="Q3" s="24" t="str">
         <f ca="1"/>
@@ -8935,7 +8940,7 @@
       </c>
       <c r="B4" s="21">
         <f ca="1">TODAY()</f>
-        <v>46086</v>
+        <v>46096</v>
       </c>
       <c r="Q4" s="24" t="str">
         <f ca="1"/>
@@ -9466,23 +9471,23 @@
       </c>
       <c r="U10" s="30" t="str">
         <f ca="1"/>
-        <v/>
-      </c>
-      <c r="V10" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="W10" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="X10" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Y10" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
+        <v>3138.9</v>
+      </c>
+      <c r="V10" s="29" t="str">
+        <f ca="1"/>
+        <v>-0.0802836297576841</v>
+      </c>
+      <c r="W10" s="29" t="str">
+        <f ca="1"/>
+        <v>-199.701758952751</v>
+      </c>
+      <c r="X10" s="29" t="str">
+        <f ca="1"/>
+        <v>-3117.99524824981</v>
+      </c>
+      <c r="Y10" s="29" t="str">
+        <f ca="1"/>
+        <v>-0.0196145797545053</v>
       </c>
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.45">
@@ -9524,23 +9529,23 @@
       </c>
       <c r="U11" s="30" t="str">
         <f ca="1"/>
-        <v/>
-      </c>
-      <c r="V11" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="W11" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="X11" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Y11" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
+        <v>2957.1</v>
+      </c>
+      <c r="V11" s="29" t="str">
+        <f ca="1"/>
+        <v>-0.189391447368421</v>
+      </c>
+      <c r="W11" s="29" t="str">
+        <f ca="1"/>
+        <v>-1091.07817610737</v>
+      </c>
+      <c r="X11" s="29" t="str">
+        <f ca="1"/>
+        <v>-4783.00750269174</v>
+      </c>
+      <c r="Y11" s="29" t="str">
+        <f ca="1"/>
+        <v>-0.0579183790499858</v>
       </c>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.45">
@@ -9562,23 +9567,23 @@
       </c>
       <c r="U12" s="30" t="str">
         <f ca="1"/>
-        <v/>
-      </c>
-      <c r="V12" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="W12" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="X12" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Y12" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
+        <v>2696</v>
+      </c>
+      <c r="V12" s="29" t="str">
+        <f ca="1"/>
+        <v>-0.197117245897734</v>
+      </c>
+      <c r="W12" s="29" t="str">
+        <f ca="1"/>
+        <v>-77.2579852931266</v>
+      </c>
+      <c r="X12" s="29" t="str">
+        <f ca="1"/>
+        <v>-2123.86037093235</v>
+      </c>
+      <c r="Y12" s="29" t="str">
+        <f ca="1"/>
+        <v>-0.0882959656420141</v>
       </c>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.45">
@@ -9651,23 +9656,23 @@
       </c>
       <c r="U13" s="30" t="str">
         <f ca="1"/>
-        <v/>
-      </c>
-      <c r="V13" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="W13" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="X13" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Y13" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
+        <v>2782.3</v>
+      </c>
+      <c r="V13" s="29" t="str">
+        <f ca="1"/>
+        <v>-0.130992910016554</v>
+      </c>
+      <c r="W13" s="29" t="str">
+        <f ca="1"/>
+        <v>661.243358811802</v>
+      </c>
+      <c r="X13" s="29" t="str">
+        <f ca="1"/>
+        <v>-706.794561541445</v>
+      </c>
+      <c r="Y13" s="29" t="str">
+        <f ca="1"/>
+        <v>0.0320103857566767</v>
       </c>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.45">
@@ -10279,20 +10284,54 @@
       <c r="C23" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D23" s="3" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="D23" ca="1">-_xll.BDH($B$2,C23,$B$3,$B$4,"DIR=H","DATES=H")</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E23" s="3"/>
-      <c r="F23" s="3"/>
-      <c r="G23" s="3"/>
-      <c r="H23" s="3"/>
-      <c r="I23" s="3"/>
-      <c r="J23" s="3"/>
-      <c r="K23" s="3"/>
-      <c r="L23" s="3"/>
-      <c r="M23" s="3"/>
-      <c r="N23" s="3"/>
+      <c r="D23" s="3" cm="1">
+        <f t="array" aca="1" ref="D23:O23" ca="1">-_xll.BDH($B$2,C23,$B$3,$B$4,"DIR=H","DATES=H")</f>
+        <v>2771.3</v>
+      </c>
+      <c r="E23" s="3">
+        <f ca="1"/>
+        <v>2830.3</v>
+      </c>
+      <c r="F23" s="3">
+        <f ca="1"/>
+        <v>3307.4</v>
+      </c>
+      <c r="G23" s="3">
+        <f ca="1"/>
+        <v>3407.2</v>
+      </c>
+      <c r="H23" s="3">
+        <f ca="1"/>
+        <v>3412.9</v>
+      </c>
+      <c r="I23" s="3">
+        <f ca="1"/>
+        <v>3648</v>
+      </c>
+      <c r="J23" s="3">
+        <f ca="1"/>
+        <v>3357.9</v>
+      </c>
+      <c r="K23" s="3">
+        <f ca="1"/>
+        <v>3201.7</v>
+      </c>
+      <c r="L23" s="3">
+        <f ca="1"/>
+        <v>3138.9</v>
+      </c>
+      <c r="M23" s="3">
+        <f ca="1"/>
+        <v>2957.1</v>
+      </c>
+      <c r="N23" s="3">
+        <f ca="1"/>
+        <v>2696</v>
+      </c>
+      <c r="O23">
+        <f ca="1"/>
+        <v>2782.3</v>
+      </c>
       <c r="Q23" s="24" t="str">
         <v>NI US EQUITY</v>
       </c>
@@ -10329,37 +10368,37 @@
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
-      <c r="H24" s="12" t="e" vm="2">
+      <c r="H24" s="12">
         <f t="shared" ref="H24:O24" ca="1" si="7">+H23/D23-1</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="I24" s="12" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J24" s="12" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K24" s="12" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L24" s="12" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M24" s="12" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N24" s="12" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O24" s="12" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
+        <v>0.23151589506729686</v>
+      </c>
+      <c r="I24" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>0.28890930290075256</v>
+      </c>
+      <c r="J24" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>1.5268791195500953E-2</v>
+      </c>
+      <c r="K24" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>-6.031345386240905E-2</v>
+      </c>
+      <c r="L24" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>-8.0283629757684105E-2</v>
+      </c>
+      <c r="M24" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>-0.18939144736842106</v>
+      </c>
+      <c r="N24" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>-0.19711724589773372</v>
+      </c>
+      <c r="O24" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>-0.13099291001655355</v>
       </c>
       <c r="Q24" s="24" t="str">
         <v>NI US EQUITY</v>
@@ -10394,21 +10433,21 @@
         <v>13</v>
       </c>
       <c r="D25" s="1"/>
-      <c r="L25" s="7" t="e">
-        <f>(L24-K24)*10000</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M25" s="7" t="e">
-        <f>(M24-L24)*10000</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N25" s="7" t="e">
-        <f>(N24-M24)*10000</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O25" s="7" t="e">
-        <f>(O24-N24)*10000</f>
-        <v>#DIV/0!</v>
+      <c r="L25" s="7">
+        <f ca="1">(L24-K24)*10000</f>
+        <v>-199.70175895275054</v>
+      </c>
+      <c r="M25" s="7">
+        <f ca="1">(M24-L24)*10000</f>
+        <v>-1091.0781761073695</v>
+      </c>
+      <c r="N25" s="7">
+        <f ca="1">(N24-M24)*10000</f>
+        <v>-77.257985293126552</v>
+      </c>
+      <c r="O25" s="7">
+        <f ca="1">(O24-N24)*10000</f>
+        <v>661.24335881180161</v>
       </c>
       <c r="Q25" s="24" t="str">
         <v>NI US EQUITY</v>
@@ -10450,21 +10489,21 @@
       <c r="I26" s="6"/>
       <c r="J26" s="6"/>
       <c r="K26" s="6"/>
-      <c r="L26" s="7" t="e">
+      <c r="L26" s="7">
         <f ca="1">(L24-H24)*10000</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M26" s="7" t="e">
-        <f>(M24-I24)*10000</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N26" s="7" t="e">
-        <f>(N24-J24)*10000</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O26" s="7" t="e">
-        <f>(O24-K24)*10000</f>
-        <v>#DIV/0!</v>
+        <v>-3117.9952482498097</v>
+      </c>
+      <c r="M26" s="7">
+        <f ca="1">(M24-I24)*10000</f>
+        <v>-4783.0075026917366</v>
+      </c>
+      <c r="N26" s="7">
+        <f ca="1">(N24-J24)*10000</f>
+        <v>-2123.8603709323465</v>
+      </c>
+      <c r="O26" s="7">
+        <f ca="1">(O24-K24)*10000</f>
+        <v>-706.79456154144509</v>
       </c>
       <c r="Q26" s="24" t="str" cm="1">
         <f t="array" ref="Q26:Y29">_xlfn.LET(
@@ -10519,21 +10558,21 @@
         <v>4</v>
       </c>
       <c r="D27" s="1"/>
-      <c r="L27" s="12" t="e">
-        <f t="shared" ref="L27:O27" si="8">L23/K23-1</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M27" s="12" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N27" s="12" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O27" s="12" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
+      <c r="L27" s="12">
+        <f t="shared" ref="L27:O27" ca="1" si="8">L23/K23-1</f>
+        <v>-1.9614579754505312E-2</v>
+      </c>
+      <c r="M27" s="12">
+        <f t="shared" ca="1" si="8"/>
+        <v>-5.7918379049985758E-2</v>
+      </c>
+      <c r="N27" s="12">
+        <f t="shared" ca="1" si="8"/>
+        <v>-8.829596564201414E-2</v>
+      </c>
+      <c r="O27" s="12">
+        <f t="shared" ca="1" si="8"/>
+        <v>3.2010385756676696E-2</v>
       </c>
       <c r="Q27" s="24" t="str">
         <v>NI US EQUITY</v>
@@ -11355,7 +11394,7 @@
       </c>
       <c r="B3" s="19">
         <f ca="1">+B4-365*3</f>
-        <v>44991</v>
+        <v>45001</v>
       </c>
       <c r="Q3" s="24" t="str">
         <f ca="1"/>
@@ -11400,7 +11439,7 @@
       </c>
       <c r="B4" s="21">
         <f ca="1">TODAY()</f>
-        <v>46086</v>
+        <v>46096</v>
       </c>
       <c r="Q4" s="24" t="str">
         <f ca="1"/>
@@ -11931,23 +11970,23 @@
       </c>
       <c r="U10" s="30" t="str">
         <f ca="1"/>
-        <v/>
-      </c>
-      <c r="V10" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="W10" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="X10" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Y10" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
+        <v>1113.5</v>
+      </c>
+      <c r="V10" s="29" t="str">
+        <f ca="1"/>
+        <v>-0.0050040210883745</v>
+      </c>
+      <c r="W10" s="29" t="str">
+        <f ca="1"/>
+        <v>690.92057675842</v>
+      </c>
+      <c r="X10" s="29" t="str">
+        <f ca="1"/>
+        <v>-70.6347667576701</v>
+      </c>
+      <c r="Y10" s="29" t="str">
+        <f ca="1"/>
+        <v>0.0207168393069941</v>
       </c>
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.45">
@@ -11989,23 +12028,23 @@
       </c>
       <c r="U11" s="30" t="str">
         <f ca="1"/>
-        <v/>
-      </c>
-      <c r="V11" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="W11" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="X11" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Y11" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
+        <v>1063.9</v>
+      </c>
+      <c r="V11" s="29" t="str">
+        <f ca="1"/>
+        <v>-0.0730963582505662</v>
+      </c>
+      <c r="W11" s="29" t="str">
+        <f ca="1"/>
+        <v>-680.923371621917</v>
+      </c>
+      <c r="X11" s="29" t="str">
+        <f ca="1"/>
+        <v>-452.315322998589</v>
+      </c>
+      <c r="Y11" s="29" t="str">
+        <f ca="1"/>
+        <v>-0.0445442299057026</v>
       </c>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.45">
@@ -12027,23 +12066,23 @@
       </c>
       <c r="U12" s="30" t="str">
         <f ca="1"/>
-        <v/>
-      </c>
-      <c r="V12" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="W12" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="X12" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Y12" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
+        <v>1049.3</v>
+      </c>
+      <c r="V12" s="29" t="str">
+        <f ca="1"/>
+        <v>-0.0398938603714888</v>
+      </c>
+      <c r="W12" s="29" t="str">
+        <f ca="1"/>
+        <v>332.024978790774</v>
+      </c>
+      <c r="X12" s="29" t="str">
+        <f ca="1"/>
+        <v>785.218853734495</v>
+      </c>
+      <c r="Y12" s="29" t="str">
+        <f ca="1"/>
+        <v>-0.0137230942757779</v>
       </c>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.45">
@@ -12116,23 +12155,23 @@
       </c>
       <c r="U13" s="30" t="str">
         <f ca="1"/>
-        <v/>
-      </c>
-      <c r="V13" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="W13" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="X13" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Y13" s="29" t="e">
-        <f ca="1"/>
-        <v>#DIV/0!</v>
+        <v>1054.4</v>
+      </c>
+      <c r="V13" s="29" t="str">
+        <f ca="1"/>
+        <v>-0.0334586121551013</v>
+      </c>
+      <c r="W13" s="29" t="str">
+        <f ca="1"/>
+        <v>64.3524821638752</v>
+      </c>
+      <c r="X13" s="29" t="str">
+        <f ca="1"/>
+        <v>406.374666091153</v>
+      </c>
+      <c r="Y13" s="29" t="str">
+        <f ca="1"/>
+        <v>0.00486038311255133</v>
       </c>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.45">
@@ -12744,20 +12783,54 @@
       <c r="C23" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D23" s="3" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="D23" ca="1">-_xll.BDH($B$2,C23,$B$3,$B$4,"DIR=H","DATES=H")</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E23" s="3"/>
-      <c r="F23" s="3"/>
-      <c r="G23" s="3"/>
-      <c r="H23" s="3"/>
-      <c r="I23" s="3"/>
-      <c r="J23" s="3"/>
-      <c r="K23" s="3"/>
-      <c r="L23" s="3"/>
-      <c r="M23" s="3"/>
-      <c r="N23" s="3"/>
+      <c r="D23" s="3" cm="1">
+        <f t="array" aca="1" ref="D23:O23" ca="1">-_xll.BDH($B$2,C23,$B$3,$B$4,"DIR=H","DATES=H")</f>
+        <v>1116.8</v>
+      </c>
+      <c r="E23" s="3">
+        <f ca="1"/>
+        <v>1180.7</v>
+      </c>
+      <c r="F23" s="3">
+        <f ca="1"/>
+        <v>1239.7</v>
+      </c>
+      <c r="G23" s="3">
+        <f ca="1"/>
+        <v>1178.2</v>
+      </c>
+      <c r="H23" s="3">
+        <f ca="1"/>
+        <v>1119.0999999999999</v>
+      </c>
+      <c r="I23" s="3">
+        <f ca="1"/>
+        <v>1147.8</v>
+      </c>
+      <c r="J23" s="3">
+        <f ca="1"/>
+        <v>1092.9000000000001</v>
+      </c>
+      <c r="K23" s="3">
+        <f ca="1"/>
+        <v>1090.9000000000001</v>
+      </c>
+      <c r="L23" s="3">
+        <f ca="1"/>
+        <v>1113.5</v>
+      </c>
+      <c r="M23" s="3">
+        <f ca="1"/>
+        <v>1063.9000000000001</v>
+      </c>
+      <c r="N23" s="3">
+        <f ca="1"/>
+        <v>1049.3</v>
+      </c>
+      <c r="O23">
+        <f ca="1"/>
+        <v>1054.4000000000001</v>
+      </c>
       <c r="Q23" s="24" t="str">
         <v>OGE US EQUITY</v>
       </c>
@@ -12794,37 +12867,37 @@
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
-      <c r="H24" s="12" t="e" vm="2">
+      <c r="H24" s="12">
         <f t="shared" ref="H24:O24" ca="1" si="7">+H23/D23-1</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="I24" s="12" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J24" s="12" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K24" s="12" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L24" s="12" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M24" s="12" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N24" s="12" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O24" s="12" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
+        <v>2.0594555873925113E-3</v>
+      </c>
+      <c r="I24" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>-2.7864825950707273E-2</v>
+      </c>
+      <c r="J24" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>-0.11841574574493829</v>
+      </c>
+      <c r="K24" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>-7.4096078764216533E-2</v>
+      </c>
+      <c r="L24" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>-5.0040210883744995E-3</v>
+      </c>
+      <c r="M24" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>-7.3096358250566151E-2</v>
+      </c>
+      <c r="N24" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>-3.9893860371488787E-2</v>
+      </c>
+      <c r="O24" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>-3.3458612155101264E-2</v>
       </c>
       <c r="Q24" s="24" t="str">
         <v>OGE US EQUITY</v>
@@ -12859,21 +12932,21 @@
         <v>13</v>
       </c>
       <c r="D25" s="1"/>
-      <c r="L25" s="7" t="e">
-        <f>(L24-K24)*10000</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M25" s="7" t="e">
-        <f>(M24-L24)*10000</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N25" s="7" t="e">
-        <f>(N24-M24)*10000</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O25" s="7" t="e">
-        <f>(O24-N24)*10000</f>
-        <v>#DIV/0!</v>
+      <c r="L25" s="7">
+        <f ca="1">(L24-K24)*10000</f>
+        <v>690.92057675842034</v>
+      </c>
+      <c r="M25" s="7">
+        <f ca="1">(M24-L24)*10000</f>
+        <v>-680.92337162191654</v>
+      </c>
+      <c r="N25" s="7">
+        <f ca="1">(N24-M24)*10000</f>
+        <v>332.02497879077362</v>
+      </c>
+      <c r="O25" s="7">
+        <f ca="1">(O24-N24)*10000</f>
+        <v>64.352482163875237</v>
       </c>
       <c r="Q25" s="24" t="str">
         <v>OGE US EQUITY</v>
@@ -12915,21 +12988,21 @@
       <c r="I26" s="6"/>
       <c r="J26" s="6"/>
       <c r="K26" s="6"/>
-      <c r="L26" s="7" t="e">
+      <c r="L26" s="7">
         <f ca="1">(L24-H24)*10000</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M26" s="7" t="e">
-        <f>(M24-I24)*10000</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N26" s="7" t="e">
-        <f>(N24-J24)*10000</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O26" s="7" t="e">
-        <f>(O24-K24)*10000</f>
-        <v>#DIV/0!</v>
+        <v>-70.634766757670107</v>
+      </c>
+      <c r="M26" s="7">
+        <f ca="1">(M24-I24)*10000</f>
+        <v>-452.31532299858878</v>
+      </c>
+      <c r="N26" s="7">
+        <f ca="1">(N24-J24)*10000</f>
+        <v>785.21885373449504</v>
+      </c>
+      <c r="O26" s="7">
+        <f ca="1">(O24-K24)*10000</f>
+        <v>406.37466609115268</v>
       </c>
       <c r="Q26" s="24" t="str" cm="1">
         <f t="array" ref="Q26:Y29">_xlfn.LET(
@@ -12984,21 +13057,21 @@
         <v>4</v>
       </c>
       <c r="D27" s="1"/>
-      <c r="L27" s="12" t="e">
-        <f t="shared" ref="L27:O27" si="8">L23/K23-1</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M27" s="12" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N27" s="12" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O27" s="12" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
+      <c r="L27" s="12">
+        <f t="shared" ref="L27:O27" ca="1" si="8">L23/K23-1</f>
+        <v>2.0716839306994084E-2</v>
+      </c>
+      <c r="M27" s="12">
+        <f t="shared" ca="1" si="8"/>
+        <v>-4.4544229905702615E-2</v>
+      </c>
+      <c r="N27" s="12">
+        <f t="shared" ca="1" si="8"/>
+        <v>-1.3723094275777892E-2</v>
+      </c>
+      <c r="O27" s="12">
+        <f t="shared" ca="1" si="8"/>
+        <v>4.8603831125513253E-3</v>
       </c>
       <c r="Q27" s="24" t="str">
         <v>OGE US EQUITY</v>

</xml_diff>